<commit_message>
Rewrite calendar captions to hook + context + CTA structure
The original captions were one-line headlines — too thin for IG/X
posts. Every feed + X caption now has the full 4-part structure
(hook → context → CTA → hashtags), the optional same-day feed posts
under each Reel slot are lightly expanded, and every reference to
a numeric "score" is removed (consistent with the comparative-rating
direction where score is derived, not typed).

Updates both the .md and the .xlsx workbook.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing/social-calendar-2026-05.xlsx
+++ b/marketing/social-calendar-2026-05.xlsx
@@ -524,7 +524,7 @@
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
@@ -587,7 +587,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
+    <row r="5" ht="110" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Setup</t>
@@ -624,7 +624,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1">
+    <row r="6" ht="110" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Setup</t>
@@ -705,7 +705,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="58" customHeight="1">
+    <row r="9" ht="110" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Mon</t>
@@ -738,11 +738,11 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Full script on the 'Reel Concepts' tab. Cross-post same cut. Optional same-day feed post: melo_social_1_home.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="58" customHeight="1">
+          <t>Full script on 'Reel Concepts' tab. Optional same-day feed post: melo_social_1_home.png — caption: "The concert app every fan needs. 🎶 Track every show, relive every year. Free on iOS — link in bio."</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="110" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Tue</t>
@@ -765,7 +765,8 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Logged my first show on Melo — setlist, vibe, who I went with, score. All in one place. Building the concert tracker I always wanted.</t>
+          <t>Logged my first show on Melo — the setlist, the vibe, who I went with, the photos. Everything about the night, in one place.
+Building the concert tracker I always wished existed. Free on iOS.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -779,7 +780,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="58" customHeight="1">
+    <row r="11" ht="110" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Wed</t>
@@ -802,7 +803,9 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Where concerts live forever.</t>
+          <t>Where concerts live forever. 🎶
+Every show you've been to — the setlist, the vibe, who you were with, the photos — kept in one place you'll actually want to revisit.
+Free on iOS. Link in bio.</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -816,7 +819,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="58" customHeight="1">
+    <row r="12" ht="110" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Thu</t>
@@ -839,12 +842,14 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Here's how Melo works ⬇️ swipe</t>
+          <t>Here's how Melo works ⬇️ swipe
+Log a show in seconds, get the setlist automatically, and watch a whole year of concerts come together. Save this for the next time someone asks what you use.
+Free on iOS. Link in bio.</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>#concertlife #livemusic #musicapp #concertdiary #musiclover</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -853,7 +858,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="58" customHeight="1">
+    <row r="13" ht="110" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Fri</t>
@@ -876,7 +881,8 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Title: "What's the show you can't stop thinking about?"</t>
+          <t>Title: "What's the show you can't stop thinking about?"
+Body: genuine question — share yours first (2-3 sentences). Mention Melo only as a footnote. NO link in body. Reply for the first 2 hrs.</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -890,7 +896,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="58" customHeight="1">
+    <row r="14" ht="110" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Daily</t>
@@ -971,7 +977,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="58" customHeight="1">
+    <row r="17" ht="110" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Mon</t>
@@ -1004,11 +1010,11 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Full script on the 'Reel Concepts' tab. Optional same-day feed post: melo_social_2_wrapped.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="58" customHeight="1">
+          <t>Full script on 'Reel Concepts' tab. Optional same-day feed post: melo_social_2_wrapped.png — caption: "Your year in music, mapped. 🗺️ Every venue you traveled to, drawn across the country. Free on iOS — link in bio."</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="110" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Tue</t>
@@ -1031,7 +1037,8 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Every show you went to — wrapped into one screen at year-end. The map, the stats, the night that defined it.</t>
+          <t>Every show you went to this year — wrapped into one screen. The map of where you traveled, the stats, the night that defined it all.
+Your concert year, the way Spotify does your listening. Free on iOS.</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1045,7 +1052,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="58" customHeight="1">
+    <row r="19" ht="110" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Wed</t>
@@ -1068,7 +1075,9 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Your year in numbers 📊 How many shows are you on track for?</t>
+          <t>Your year in numbers 📊
+Shows seen, venues visited, miles traveled, songs heard live — Melo counts it all while you just go to concerts.
+How many shows are you on track for this year? Tell me below ⬇️</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1082,7 +1091,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="58" customHeight="1">
+    <row r="20" ht="110" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Thu</t>
@@ -1105,7 +1114,9 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>How long is your concert streak? 🔥</t>
+          <t>How long is your concert streak? 🔥
+Melo tracks how many months in a row you've caught a show — and quietly dares you not to break it.
+Drop your current streak in the comments ⬇️</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1119,7 +1130,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="58" customHeight="1">
+    <row r="21" ht="110" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Fri</t>
@@ -1142,7 +1153,8 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Title: "How do you remember which set was actually good 6 months later?"</t>
+          <t>Title: "How do you remember which set was actually good 6 months later?"
+Body: genuine question, your answer first, Melo as footnote, no link in body.</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1156,7 +1168,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="58" customHeight="1">
+    <row r="22" ht="110" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Daily</t>
@@ -1237,7 +1249,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="58" customHeight="1">
+    <row r="25" ht="110" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Mon</t>
@@ -1270,11 +1282,11 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Full script on the 'Reel Concepts' tab. Optional same-day feed post: melo_fixed_03_setlist.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="58" customHeight="1">
+          <t>Full script on 'Reel Concepts' tab. Optional same-day feed post: melo_fixed_03_setlist.png — caption: "Never forget a setlist. 🎤 Melo pulls the full setlist for every show automatically — zero typing. Free on iOS — link in bio."</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="110" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Tue</t>
@@ -1297,7 +1309,8 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Every show gets its own page — photos, the full setlist, the vibe of the night, your score.</t>
+          <t>Every show gets its own page in Melo — your photos, the full setlist, the vibe of the night, a home for everything you'll want to remember.
+Your concert history, finally kept properly. Free on iOS.</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -1311,7 +1324,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="58" customHeight="1">
+    <row r="27" ht="110" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Wed</t>
@@ -1334,7 +1347,9 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>What was the vibe? 👀 Euphoric, intimate, rowdy, chill…</t>
+          <t>What was the vibe? 👀
+Euphoric, intimate, rowdy, chill, transcendent — Melo lets you tag how every show actually *felt*, not just who played it.
+What's the vibe of the best show you've ever been to? ⬇️</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -1348,7 +1363,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="58" customHeight="1">
+    <row r="28" ht="110" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Thu</t>
@@ -1371,12 +1386,14 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>→ For everyone asking how it works</t>
+          <t>→ For everyone asking how it works
+Swipe through the whole thing — logging, vibes, your year wrapped. Then go start your own concert history.
+Free on iOS. Link in bio.</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>#concertlife #livemusic #musicapp #concertdiary #musiclover</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -1385,7 +1402,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="58" customHeight="1">
+    <row r="29" ht="110" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Fri</t>
@@ -1422,7 +1439,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="58" customHeight="1">
+    <row r="30" ht="110" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Daily</t>
@@ -1503,7 +1520,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="58" customHeight="1">
+    <row r="33" ht="110" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
           <t>Mon</t>
@@ -1536,11 +1553,11 @@
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>Your one founder reel. Full script on the 'Reel Concepts' tab. Optional same-day feed post: melo_onbrand_04_fixed.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="58" customHeight="1">
+          <t>Your one founder reel. Full script on 'Reel Concepts' tab. Optional same-day feed post: melo_onbrand_04_fixed.png — caption: "Festival szn. Track every set. 🎪 Every artist, every stage, every weekend — logged. Free on iOS — link in bio."</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="110" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
           <t>Tue</t>
@@ -1563,7 +1580,8 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Concerts are better with people. Melo logs who you went with — so years later you remember the night AND the crew.</t>
+          <t>Concerts are better with people. Melo logs who you went with on every show — so years later you remember the night AND the crew you saw it with.
+Tag your concert person. Free on iOS.</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -1577,7 +1595,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="58" customHeight="1">
+    <row r="35" ht="110" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
           <t>Wed</t>
@@ -1600,7 +1618,9 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>The shows you've seen, never forgotten.</t>
+          <t>The shows you've seen, never forgotten. 🎶
+Years from now you won't remember the date — but you'll remember the room, the crowd, the moment. Melo keeps all of it.
+Free on iOS. Link in bio.</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -1614,7 +1634,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="58" customHeight="1">
+    <row r="36" ht="110" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
           <t>Thu</t>
@@ -1637,7 +1657,9 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Tickets in pocket. App open. Memory secured.</t>
+          <t>Tickets in pocket. App open. Memory secured. 🎟️
+Log the show before you even leave the venue — the setlist, the vibe, the photos, the whole night.
+Free on iOS. Link in bio.</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -1651,7 +1673,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="58" customHeight="1">
+    <row r="37" ht="110" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Fri</t>
@@ -1674,7 +1696,8 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Title: "The best concert you've ever been to — go."</t>
+          <t>Title: "The best concert you've ever been to — go."
+Body: genuine question, your answer first, Melo as a footnote, no link in body.</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -1688,7 +1711,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="58" customHeight="1">
+    <row r="38" ht="110" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
           <t>Daily</t>

</xml_diff>